<commit_message>
Same-breath sweep for the A1 refinement (Sunny's catch): contract §7 checklist, KG1 registry, L1 code map
INTAKE-8/9 added to the §7 list; registration rule row in
Rules_to_Checks (+ stale ReadMe open-items cleared); code map:
validate_extract cites 0..9, new kg1_intake.apply_registration
(the only path that mints a db node). One refusal fixture noted
to author.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BAgZi4RCB3bWFG5MSWcW8V
</commit_message>
<xml_diff>
--- a/AIVIA_Design/L1_Code_Structure_Map_DRAFT.xlsx
+++ b/AIVIA_Design/L1_Code_Structure_Map_DRAFT.xlsx
@@ -681,7 +681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -930,7 +930,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>INTAKE-0..7; LC-F5 atomicity decided BEFORE any write</t>
+          <t>INTAKE-0..9 (8: unregistered db refused; 9: declared-vs-captured agreement); LC-F5 atomicity decided BEFORE any write</t>
         </is>
       </c>
     </row>
@@ -1390,6 +1390,33 @@
       <c r="E26" s="2" t="inlineStr">
         <is>
           <t>the ONLY import surface for Level 2 (plank); B3 on every result</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>kg1_intake.apply_registration</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>RegistrationPrereq (DBA-completed: db, server, dba team, sources)</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>db node + layer-3 dba responsibility</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>KG1 db mint + LC3-C (responsibility)</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>A1 refined: runs BEFORE any extract intake; the only path that mints a db node</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Source defined and grounded (Sunny's SSMS deciding example): registration's schema mapping, identity component, never stored twice
The label SSMS never shows: which system put a schema's tables
there — DBA-declared in the registration prereq's schema mapping;
since A2 the first component of identity, no second stored field.
Doc, contract §12 (+INTAKE-8 fold), F1 (registration schema_sources
+ expected schemas cleaned), KG1 registry, and code map moved in
the same breath.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BAgZi4RCB3bWFG5MSWcW8V
</commit_message>
<xml_diff>
--- a/AIVIA_Design/L1_Code_Structure_Map_DRAFT.xlsx
+++ b/AIVIA_Design/L1_Code_Structure_Map_DRAFT.xlsx
@@ -1401,7 +1401,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>RegistrationPrereq (DBA-completed: db, server, dba team, sources)</t>
+          <t>RegistrationPrereq (DBA-completed: db, server, dba team, sources, schema-&gt;source mapping)</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>A1 refined: runs BEFORE any extract intake; the only path that mints a db node</t>
+          <t>A1 refined + source ruling: runs BEFORE any intake; the only path that mints a db node; the mapping is where source identities originate</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
pk is declared data (Sunny's CLARITY_TBL_PK fact): extract part 3b, INTAKE-10 integrity, prose rule retired
The pk metadata table joins the source pack; every table must
carry declared pk rows (named refusal otherwise); pk gap list
retires as structurally empty; grain stays opportunistic. F1 gains
pk.csv in both snapshots, all seven pks filled, referenced_keys
expectations added (pk vs referenced-key visibly differ on
ENCOUNTER_DX). Registry, code map, contract, doc, Protected notes
moved in the same breath. Two confirms for Sunny: composite-pk
ordinal column; live census of tables without pk rows.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BAgZi4RCB3bWFG5MSWcW8V
</commit_message>
<xml_diff>
--- a/AIVIA_Design/L1_Code_Structure_Map_DRAFT.xlsx
+++ b/AIVIA_Design/L1_Code_Structure_Map_DRAFT.xlsx
@@ -930,7 +930,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>INTAKE-0..9 (8: unregistered db refused; 9: declared-vs-captured agreement); LC-F5 atomicity decided BEFORE any write</t>
+          <t>INTAKE-0..10 (8 unregistered db; 9 declared-vs-captured; 10 pk integrity); LC-F5 atomicity decided BEFORE any write</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>business_name? grain? pk_columns? + gap rows</t>
+          <t>business_name? grain? + gap rows (pk phrase RETIRED 2026-09-05)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">

</xml_diff>